<commit_message>
good version only for binary
</commit_message>
<xml_diff>
--- a/inst/extdata/clinical_studies_data.xlsx
+++ b/inst/extdata/clinical_studies_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkStation\Products\AIMetaAnalysis\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8D697B-6E2F-42AD-9929-8C936EB1E5A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E4EABC-35C8-4028-A4E5-CCDF23C486BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{E48AEDA6-24C4-4F19-8C79-FEB57B06AF66}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="continuous" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">binary_data!$A$1:$Y$786</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">binary_data!$A$1:$Y$800</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7867" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8001" uniqueCount="269">
   <si>
     <t>study</t>
   </si>
@@ -1232,6 +1232,25 @@
     <t>moreEqualThan_1_Percent</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
+  <si>
+    <t>Neoadjuvant_cycles</t>
+  </si>
+  <si>
+    <t>Neoadjuvant_cycles</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Overall</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>3 Cycles</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>4 Cycles</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1293,7 +1312,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1348,6 +1367,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1363,7 +1388,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1405,6 +1430,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1926,7 +1955,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{631E57DE-EBE0-4137-B3CA-3E2E983F6363}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:AN786"/>
+  <dimension ref="A1:AN800"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="5"/>
@@ -37267,7 +37296,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="718" spans="1:28" hidden="1" x14ac:dyDescent="0.35">
+    <row r="718" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A718" s="5" t="s">
         <v>58</v>
       </c>
@@ -37316,7 +37345,7 @@
         <v>GOOD</v>
       </c>
     </row>
-    <row r="719" spans="1:28" hidden="1" x14ac:dyDescent="0.35">
+    <row r="719" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A719" s="5" t="s">
         <v>58</v>
       </c>
@@ -38312,7 +38341,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="740" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="740" spans="1:40" hidden="1" x14ac:dyDescent="0.35">
       <c r="A740" s="5" t="s">
         <v>58</v>
       </c>
@@ -38361,7 +38390,7 @@
         <v>GOOD</v>
       </c>
     </row>
-    <row r="741" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="741" spans="1:40" hidden="1" x14ac:dyDescent="0.35">
       <c r="A741" s="5" t="s">
         <v>58</v>
       </c>
@@ -38407,7 +38436,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="742" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="742" spans="1:40" hidden="1" x14ac:dyDescent="0.35">
       <c r="A742" s="5" t="s">
         <v>58</v>
       </c>
@@ -38456,7 +38485,7 @@
         <v>GOOD</v>
       </c>
     </row>
-    <row r="743" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="743" spans="1:40" hidden="1" x14ac:dyDescent="0.35">
       <c r="A743" s="5" t="s">
         <v>58</v>
       </c>
@@ -40323,8 +40352,664 @@
         <v>249</v>
       </c>
     </row>
+    <row r="787" spans="1:16" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A787" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C787" s="21">
+        <v>1030</v>
+      </c>
+      <c r="D787" s="21">
+        <v>1</v>
+      </c>
+      <c r="E787" s="21" t="s">
+        <v>210</v>
+      </c>
+      <c r="F787" s="21">
+        <v>2022</v>
+      </c>
+      <c r="G787" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H787" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="I787" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J787" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K787" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="M787" s="21" t="s">
+        <v>266</v>
+      </c>
+      <c r="N787" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="O787" s="21">
+        <f>O10</f>
+        <v>3.9380000000000002</v>
+      </c>
+      <c r="P787" s="21">
+        <f>P10</f>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="788" spans="1:16" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A788" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C788" s="21">
+        <v>1030</v>
+      </c>
+      <c r="D788" s="21">
+        <v>1</v>
+      </c>
+      <c r="E788" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="F788" s="21">
+        <v>2022</v>
+      </c>
+      <c r="G788" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H788" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="I788" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J788" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K788" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="M788" s="21" t="s">
+        <v>266</v>
+      </c>
+      <c r="N788" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="O788" s="21">
+        <f>O11</f>
+        <v>42.96</v>
+      </c>
+      <c r="P788" s="21">
+        <f>P11</f>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="789" spans="1:16" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A789" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B789" s="5"/>
+      <c r="C789" s="5"/>
+      <c r="D789" s="5"/>
+      <c r="E789" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="F789" s="5">
+        <v>2023</v>
+      </c>
+      <c r="G789" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="H789" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="I789" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J789" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K789" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="M789" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N789" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="O789" s="21">
+        <f>O716</f>
+        <v>21</v>
+      </c>
+      <c r="P789" s="21">
+        <f>P716</f>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="790" spans="1:16" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A790" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B790" s="5"/>
+      <c r="C790" s="5"/>
+      <c r="D790" s="5"/>
+      <c r="E790" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="F790" s="5">
+        <v>2023</v>
+      </c>
+      <c r="G790" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="H790" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="I790" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J790" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K790" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="M790" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N790" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="O790" s="21">
+        <f>O717</f>
+        <v>2</v>
+      </c>
+      <c r="P790" s="21">
+        <f>P717</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="791" spans="1:16" s="21" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A791" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B791" s="5"/>
+      <c r="C791" s="5"/>
+      <c r="D791" s="5"/>
+      <c r="E791" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="F791" s="5">
+        <v>2023</v>
+      </c>
+      <c r="G791" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H791" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I791" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J791" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K791" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="M791" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="N791" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="O791" s="21">
+        <f>O718</f>
+        <v>14.017999999999999</v>
+      </c>
+      <c r="P791" s="21">
+        <f>P718</f>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="792" spans="1:16" s="21" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A792" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B792" s="5"/>
+      <c r="C792" s="5"/>
+      <c r="D792" s="5"/>
+      <c r="E792" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="F792" s="5">
+        <v>2023</v>
+      </c>
+      <c r="G792" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H792" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I792" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J792" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K792" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="M792" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="N792" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="O792" s="21">
+        <f>O719</f>
+        <v>4.0049999999999999</v>
+      </c>
+      <c r="P792" s="21">
+        <f>P719</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="793" spans="1:16" s="21" customFormat="1" ht="42.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A793" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C793" s="21">
+        <v>1120</v>
+      </c>
+      <c r="D793" s="21">
+        <v>5</v>
+      </c>
+      <c r="E793" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="F793" s="21">
+        <v>2024</v>
+      </c>
+      <c r="G793" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H793" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="I793" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J793" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K793" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L793" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M793" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N793" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="O793" s="21">
+        <f>O714</f>
+        <v>50.096000000000004</v>
+      </c>
+      <c r="P793" s="21">
+        <f>P714</f>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="794" spans="1:16" s="21" customFormat="1" ht="42.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A794" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C794" s="21">
+        <v>1120</v>
+      </c>
+      <c r="D794" s="21">
+        <v>5</v>
+      </c>
+      <c r="E794" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="F794" s="21">
+        <v>2024</v>
+      </c>
+      <c r="G794" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H794" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="I794" s="21" t="s">
+        <v>264</v>
+      </c>
+      <c r="J794" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="K794" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L794" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M794" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N794" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="O794" s="21">
+        <f>O715</f>
+        <v>2.02</v>
+      </c>
+      <c r="P794" s="21">
+        <f>P715</f>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="795" spans="1:16" s="21" customFormat="1" ht="42.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A795" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C795" s="21">
+        <v>1130</v>
+      </c>
+      <c r="D795" s="21">
+        <v>3</v>
+      </c>
+      <c r="E795" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F795" s="21">
+        <v>2023</v>
+      </c>
+      <c r="G795" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H795" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="I795" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J795" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="K795" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L795" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M795" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N795" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="O795" s="21">
+        <f>O8</f>
+        <v>62.951999999999998</v>
+      </c>
+      <c r="P795" s="21">
+        <f>P8</f>
+        <v>366</v>
+      </c>
+    </row>
+    <row r="796" spans="1:16" s="21" customFormat="1" ht="12.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A796" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C796" s="21">
+        <v>1130</v>
+      </c>
+      <c r="D796" s="21">
+        <v>3</v>
+      </c>
+      <c r="E796" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F796" s="21">
+        <v>2023</v>
+      </c>
+      <c r="G796" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H796" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="I796" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J796" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="K796" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L796" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M796" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N796" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="O796" s="21">
+        <f>O9</f>
+        <v>16.082000000000001</v>
+      </c>
+      <c r="P796" s="21">
+        <f>P9</f>
+        <v>374</v>
+      </c>
+    </row>
+    <row r="797" spans="1:16" s="21" customFormat="1" ht="42.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A797" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C797" s="21">
+        <v>1020</v>
+      </c>
+      <c r="D797" s="21">
+        <v>2</v>
+      </c>
+      <c r="E797" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="F797" s="21">
+        <v>2024</v>
+      </c>
+      <c r="G797" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H797" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="I797" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J797" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="K797" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L797" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="M797" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="N797" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="O797" s="21">
+        <f>O12</f>
+        <v>57.936999999999998</v>
+      </c>
+      <c r="P797" s="21">
+        <f>P12</f>
+        <v>229</v>
+      </c>
+    </row>
+    <row r="798" spans="1:16" s="21" customFormat="1" ht="42.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A798" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C798" s="21">
+        <v>1020</v>
+      </c>
+      <c r="D798" s="21">
+        <v>2</v>
+      </c>
+      <c r="E798" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="F798" s="21">
+        <v>2024</v>
+      </c>
+      <c r="G798" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H798" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="I798" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J798" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="K798" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L798" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="M798" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="N798" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="O798" s="21">
+        <f>O13</f>
+        <v>10.904000000000002</v>
+      </c>
+      <c r="P798" s="21">
+        <f>P13</f>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="799" spans="1:16" s="21" customFormat="1" ht="42.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A799" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C799" s="21">
+        <v>1100</v>
+      </c>
+      <c r="D799" s="21">
+        <v>4</v>
+      </c>
+      <c r="E799" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="F799" s="21">
+        <v>2024</v>
+      </c>
+      <c r="G799" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H799" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="I799" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J799" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="K799" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L799" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M799" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N799" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="O799" s="21">
+        <f>O30</f>
+        <v>72</v>
+      </c>
+      <c r="P799" s="21">
+        <f>P30</f>
+        <v>397</v>
+      </c>
+    </row>
+    <row r="800" spans="1:16" s="21" customFormat="1" ht="42.45" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A800" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C800" s="21">
+        <v>1100</v>
+      </c>
+      <c r="D800" s="21">
+        <v>4</v>
+      </c>
+      <c r="E800" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="F800" s="21">
+        <v>2024</v>
+      </c>
+      <c r="G800" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H800" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="I800" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="J800" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="K800" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="L800" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M800" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N800" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="O800" s="21">
+        <f>O31</f>
+        <v>16</v>
+      </c>
+      <c r="P800" s="21">
+        <f>P31</f>
+        <v>400</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y786" xr:uid="{631E57DE-EBE0-4137-B3CA-3E2E983F6363}">
+  <autoFilter ref="A1:Y800" xr:uid="{631E57DE-EBE0-4137-B3CA-3E2E983F6363}">
     <filterColumn colId="4">
       <filters>
         <filter val="TD-FOREKNOW"/>
@@ -40337,7 +41022,8 @@
     </filterColumn>
     <filterColumn colId="8">
       <filters>
-        <filter val="PD-L1 expression level"/>
+        <filter val="Neoadjuvant_cycles"/>
+        <filter val="Overall"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>